<commit_message>
analise de variância atualizadas
</commit_message>
<xml_diff>
--- a/data-raw/dadoscpfl.xlsx
+++ b/data-raw/dadoscpfl.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a61b52e7261446ee/AA TOTONHO TRABALHO/HIDRELÉTRICAS/CPFL incorporação/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\macrofitas-cpfl\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="8_{D665FB8D-F563-4CD1-8B90-C887F7EE3771}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EBDAC0C4-82D4-404D-B57D-0AF38C92DEB6}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7495712A-55D4-432F-A9C8-BE4495DA54C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{49060A0B-62BF-4EE6-B69F-8F435598AA6F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{49060A0B-62BF-4EE6-B69F-8F435598AA6F}"/>
   </bookViews>
   <sheets>
     <sheet name="Composição química macrófitas" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="50">
   <si>
     <t>Amostra</t>
   </si>
@@ -177,9 +177,6 @@
   </si>
   <si>
     <t>20 t/ha</t>
-  </si>
-  <si>
-    <t>22 t/ha</t>
   </si>
   <si>
     <t>05 t/ha</t>
@@ -443,10 +440,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -767,12 +760,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{591271F4-E98E-471E-81E6-ADD714D6BD01}">
   <dimension ref="A1:Q37"/>
-  <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.21875" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="9.23046875" style="3"/>
+    <col min="1" max="16384" width="9.21875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="E1" s="35" t="s">
         <v>22</v>
       </c>
@@ -789,7 +782,7 @@
       <c r="P1" s="35"/>
       <c r="Q1" s="35"/>
     </row>
-    <row r="2" spans="1:17" s="5" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:17" s="5" customFormat="1" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4"/>
       <c r="B2" s="7" t="s">
         <v>0</v>
@@ -840,7 +833,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="6">
         <v>43132</v>
       </c>
@@ -893,7 +886,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="6">
         <v>43132</v>
       </c>
@@ -946,7 +939,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="6">
         <v>43132</v>
       </c>
@@ -999,7 +992,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="6">
         <v>43132</v>
       </c>
@@ -1052,7 +1045,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="6">
         <v>43132</v>
       </c>
@@ -1105,7 +1098,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="6">
         <v>43132</v>
       </c>
@@ -1158,7 +1151,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="6">
         <v>43132</v>
       </c>
@@ -1211,7 +1204,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="6">
         <v>43132</v>
       </c>
@@ -1264,7 +1257,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="6">
         <v>43132</v>
       </c>
@@ -1317,7 +1310,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="6">
         <v>43132</v>
       </c>
@@ -1370,7 +1363,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="6">
         <v>43132</v>
       </c>
@@ -1423,7 +1416,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="6">
         <v>43132</v>
       </c>
@@ -1476,7 +1469,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="6">
         <v>43132</v>
       </c>
@@ -1529,7 +1522,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="6">
         <v>43132</v>
       </c>
@@ -1582,7 +1575,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="17" spans="1:17" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:17" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="14">
         <v>43132</v>
       </c>
@@ -1635,7 +1628,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="6">
         <v>43252</v>
       </c>
@@ -1688,7 +1681,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="6">
         <v>43252</v>
       </c>
@@ -1741,7 +1734,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="6">
         <v>43252</v>
       </c>
@@ -1794,7 +1787,7 @@
         <v>6.9</v>
       </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="6">
         <v>43252</v>
       </c>
@@ -1847,7 +1840,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="6">
         <v>43252</v>
       </c>
@@ -1900,7 +1893,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="6">
         <v>43252</v>
       </c>
@@ -1953,7 +1946,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="6">
         <v>43252</v>
       </c>
@@ -2006,7 +1999,7 @@
         <v>19.5</v>
       </c>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="6">
         <v>43252</v>
       </c>
@@ -2059,7 +2052,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="6">
         <v>43252</v>
       </c>
@@ -2112,7 +2105,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="6">
         <v>43252</v>
       </c>
@@ -2165,7 +2158,7 @@
         <v>16.899999999999999</v>
       </c>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A28" s="6">
         <v>43252</v>
       </c>
@@ -2218,7 +2211,7 @@
         <v>33.1</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="6">
         <v>43252</v>
       </c>
@@ -2271,7 +2264,7 @@
         <v>27.8</v>
       </c>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A30" s="6">
         <v>43252</v>
       </c>
@@ -2324,7 +2317,7 @@
         <v>15.5</v>
       </c>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="6">
         <v>43252</v>
       </c>
@@ -2377,7 +2370,7 @@
         <v>23.8</v>
       </c>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="6">
         <v>43252</v>
       </c>
@@ -2430,7 +2423,7 @@
         <v>17.3</v>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="6">
         <v>43252</v>
       </c>
@@ -2483,7 +2476,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="6">
         <v>43252</v>
       </c>
@@ -2536,7 +2529,7 @@
         <v>16.399999999999999</v>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="6">
         <v>43252</v>
       </c>
@@ -2589,7 +2582,7 @@
         <v>14.4</v>
       </c>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="6">
         <v>43252</v>
       </c>
@@ -2642,7 +2635,7 @@
         <v>14.4</v>
       </c>
     </row>
-    <row r="37" spans="1:17" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:17" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="14">
         <v>43252</v>
       </c>
@@ -2709,17 +2702,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17C4B281-7CCE-4DF9-9F04-7DA15B43C9D7}">
   <dimension ref="A1:I41"/>
-  <sheetFormatPr defaultRowHeight="16" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="7" max="7" width="9.23046875" customWidth="1"/>
+    <col min="7" max="7" width="9.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="33" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B1" s="33" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C1" s="33" t="s">
         <v>23</v>
@@ -2728,7 +2721,7 @@
         <v>39</v>
       </c>
       <c r="E1" s="33" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F1" s="33" t="s">
         <v>40</v>
@@ -2737,7 +2730,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="33" t="s">
         <v>42</v>
       </c>
@@ -2759,7 +2752,7 @@
       </c>
       <c r="I2" s="33"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="33" t="s">
         <v>42</v>
       </c>
@@ -2780,7 +2773,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="33" t="s">
         <v>42</v>
       </c>
@@ -2801,7 +2794,7 @@
         <v>1.02</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="33" t="s">
         <v>42</v>
       </c>
@@ -2822,12 +2815,12 @@
         <v>1.06</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="33" t="s">
         <v>16</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C6" s="34">
         <v>1</v>
@@ -2846,12 +2839,12 @@
       </c>
       <c r="I6" s="33"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="33" t="s">
         <v>16</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C7" s="34">
         <v>2</v>
@@ -2869,12 +2862,12 @@
         <v>0.89</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="33" t="s">
         <v>16</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C8" s="34">
         <v>3</v>
@@ -2892,12 +2885,12 @@
         <v>0.91</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="33" t="s">
         <v>16</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C9" s="34">
         <v>4</v>
@@ -2915,7 +2908,7 @@
         <v>0.95823999999999954</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="33" t="s">
         <v>16</v>
       </c>
@@ -2939,7 +2932,7 @@
       </c>
       <c r="I10" s="33"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="33" t="s">
         <v>16</v>
       </c>
@@ -2962,7 +2955,7 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="33" t="s">
         <v>16</v>
       </c>
@@ -2985,7 +2978,7 @@
         <v>1.32</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="33" t="s">
         <v>16</v>
       </c>
@@ -3008,7 +3001,7 @@
         <v>1.1134399999999998</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="33" t="s">
         <v>16</v>
       </c>
@@ -3032,7 +3025,7 @@
       </c>
       <c r="I14" s="33"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="33" t="s">
         <v>16</v>
       </c>
@@ -3055,7 +3048,7 @@
         <v>0.98</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="33" t="s">
         <v>16</v>
       </c>
@@ -3078,12 +3071,12 @@
         <v>1.21</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="33" t="s">
         <v>16</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C17" s="34">
         <v>4</v>
@@ -3101,12 +3094,12 @@
         <v>1.3040799999999999</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="33" t="s">
         <v>18</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C18" s="34">
         <v>1</v>
@@ -3125,12 +3118,12 @@
       </c>
       <c r="I18" s="33"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="33" t="s">
         <v>18</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C19" s="34">
         <v>2</v>
@@ -3148,12 +3141,12 @@
         <v>1.74</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="33" t="s">
         <v>18</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C20" s="34">
         <v>3</v>
@@ -3171,12 +3164,12 @@
         <v>1.49</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="33" t="s">
         <v>18</v>
       </c>
       <c r="B21" s="33" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C21" s="34">
         <v>4</v>
@@ -3194,7 +3187,7 @@
         <v>1.5225600000000004</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="33" t="s">
         <v>18</v>
       </c>
@@ -3218,7 +3211,7 @@
       </c>
       <c r="I22" s="33"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="33" t="s">
         <v>18</v>
       </c>
@@ -3241,7 +3234,7 @@
         <v>1.55</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="33" t="s">
         <v>18</v>
       </c>
@@ -3264,7 +3257,7 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="33" t="s">
         <v>18</v>
       </c>
@@ -3287,7 +3280,7 @@
         <v>1.5024800000000003</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="33" t="s">
         <v>18</v>
       </c>
@@ -3311,7 +3304,7 @@
       </c>
       <c r="I26" s="33"/>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="33" t="s">
         <v>18</v>
       </c>
@@ -3334,7 +3327,7 @@
         <v>1.51</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="33" t="s">
         <v>18</v>
       </c>
@@ -3357,7 +3350,7 @@
         <v>1.72</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="33" t="s">
         <v>18</v>
       </c>
@@ -3380,12 +3373,12 @@
         <v>1.6856000000000009</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="33" t="s">
         <v>19</v>
       </c>
       <c r="B30" s="33" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C30" s="34">
         <v>1</v>
@@ -3404,12 +3397,12 @@
       </c>
       <c r="I30" s="33"/>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="33" t="s">
         <v>19</v>
       </c>
       <c r="B31" s="33" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C31" s="34">
         <v>2</v>
@@ -3427,12 +3420,12 @@
         <v>1.74</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="33" t="s">
         <v>19</v>
       </c>
       <c r="B32" s="33" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C32" s="34">
         <v>3</v>
@@ -3450,12 +3443,12 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="33" t="s">
         <v>19</v>
       </c>
       <c r="B33" s="33" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C33" s="34">
         <v>4</v>
@@ -3473,7 +3466,7 @@
         <v>1.7875999999999985</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="33" t="s">
         <v>19</v>
       </c>
@@ -3496,7 +3489,7 @@
         <v>1.63</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="33" t="s">
         <v>19</v>
       </c>
@@ -3520,7 +3513,7 @@
       </c>
       <c r="I35" s="33"/>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="33" t="s">
         <v>19</v>
       </c>
@@ -3543,7 +3536,7 @@
         <v>1.48</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="33" t="s">
         <v>19</v>
       </c>
@@ -3566,7 +3559,7 @@
         <v>1.928799999999999</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="33" t="s">
         <v>19</v>
       </c>
@@ -3590,7 +3583,7 @@
       </c>
       <c r="I38" s="33"/>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="33" t="s">
         <v>19</v>
       </c>
@@ -3613,7 +3606,7 @@
         <v>1.67</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="33" t="s">
         <v>19</v>
       </c>
@@ -3636,7 +3629,7 @@
         <v>1.38</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="33" t="s">
         <v>19</v>
       </c>
@@ -3671,142 +3664,142 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F1885F8-2F2E-49F4-83AE-FDFEDBECDBCF}">
   <dimension ref="A1:X52"/>
-  <sheetFormatPr defaultRowHeight="16" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.69140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.921875" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="25" width="7.3046875" style="1" customWidth="1"/>
-    <col min="26" max="256" width="9.23046875" style="1"/>
-    <col min="257" max="281" width="7.3046875" style="1" customWidth="1"/>
-    <col min="282" max="512" width="9.23046875" style="1"/>
-    <col min="513" max="537" width="7.3046875" style="1" customWidth="1"/>
-    <col min="538" max="768" width="9.23046875" style="1"/>
-    <col min="769" max="793" width="7.3046875" style="1" customWidth="1"/>
-    <col min="794" max="1024" width="9.23046875" style="1"/>
-    <col min="1025" max="1049" width="7.3046875" style="1" customWidth="1"/>
-    <col min="1050" max="1280" width="9.23046875" style="1"/>
-    <col min="1281" max="1305" width="7.3046875" style="1" customWidth="1"/>
-    <col min="1306" max="1536" width="9.23046875" style="1"/>
-    <col min="1537" max="1561" width="7.3046875" style="1" customWidth="1"/>
-    <col min="1562" max="1792" width="9.23046875" style="1"/>
-    <col min="1793" max="1817" width="7.3046875" style="1" customWidth="1"/>
-    <col min="1818" max="2048" width="9.23046875" style="1"/>
-    <col min="2049" max="2073" width="7.3046875" style="1" customWidth="1"/>
-    <col min="2074" max="2304" width="9.23046875" style="1"/>
-    <col min="2305" max="2329" width="7.3046875" style="1" customWidth="1"/>
-    <col min="2330" max="2560" width="9.23046875" style="1"/>
-    <col min="2561" max="2585" width="7.3046875" style="1" customWidth="1"/>
-    <col min="2586" max="2816" width="9.23046875" style="1"/>
-    <col min="2817" max="2841" width="7.3046875" style="1" customWidth="1"/>
-    <col min="2842" max="3072" width="9.23046875" style="1"/>
-    <col min="3073" max="3097" width="7.3046875" style="1" customWidth="1"/>
-    <col min="3098" max="3328" width="9.23046875" style="1"/>
-    <col min="3329" max="3353" width="7.3046875" style="1" customWidth="1"/>
-    <col min="3354" max="3584" width="9.23046875" style="1"/>
-    <col min="3585" max="3609" width="7.3046875" style="1" customWidth="1"/>
-    <col min="3610" max="3840" width="9.23046875" style="1"/>
-    <col min="3841" max="3865" width="7.3046875" style="1" customWidth="1"/>
-    <col min="3866" max="4096" width="9.23046875" style="1"/>
-    <col min="4097" max="4121" width="7.3046875" style="1" customWidth="1"/>
-    <col min="4122" max="4352" width="9.23046875" style="1"/>
-    <col min="4353" max="4377" width="7.3046875" style="1" customWidth="1"/>
-    <col min="4378" max="4608" width="9.23046875" style="1"/>
-    <col min="4609" max="4633" width="7.3046875" style="1" customWidth="1"/>
-    <col min="4634" max="4864" width="9.23046875" style="1"/>
-    <col min="4865" max="4889" width="7.3046875" style="1" customWidth="1"/>
-    <col min="4890" max="5120" width="9.23046875" style="1"/>
-    <col min="5121" max="5145" width="7.3046875" style="1" customWidth="1"/>
-    <col min="5146" max="5376" width="9.23046875" style="1"/>
-    <col min="5377" max="5401" width="7.3046875" style="1" customWidth="1"/>
-    <col min="5402" max="5632" width="9.23046875" style="1"/>
-    <col min="5633" max="5657" width="7.3046875" style="1" customWidth="1"/>
-    <col min="5658" max="5888" width="9.23046875" style="1"/>
-    <col min="5889" max="5913" width="7.3046875" style="1" customWidth="1"/>
-    <col min="5914" max="6144" width="9.23046875" style="1"/>
-    <col min="6145" max="6169" width="7.3046875" style="1" customWidth="1"/>
-    <col min="6170" max="6400" width="9.23046875" style="1"/>
-    <col min="6401" max="6425" width="7.3046875" style="1" customWidth="1"/>
-    <col min="6426" max="6656" width="9.23046875" style="1"/>
-    <col min="6657" max="6681" width="7.3046875" style="1" customWidth="1"/>
-    <col min="6682" max="6912" width="9.23046875" style="1"/>
-    <col min="6913" max="6937" width="7.3046875" style="1" customWidth="1"/>
-    <col min="6938" max="7168" width="9.23046875" style="1"/>
-    <col min="7169" max="7193" width="7.3046875" style="1" customWidth="1"/>
-    <col min="7194" max="7424" width="9.23046875" style="1"/>
-    <col min="7425" max="7449" width="7.3046875" style="1" customWidth="1"/>
-    <col min="7450" max="7680" width="9.23046875" style="1"/>
-    <col min="7681" max="7705" width="7.3046875" style="1" customWidth="1"/>
-    <col min="7706" max="7936" width="9.23046875" style="1"/>
-    <col min="7937" max="7961" width="7.3046875" style="1" customWidth="1"/>
-    <col min="7962" max="8192" width="9.23046875" style="1"/>
-    <col min="8193" max="8217" width="7.3046875" style="1" customWidth="1"/>
-    <col min="8218" max="8448" width="9.23046875" style="1"/>
-    <col min="8449" max="8473" width="7.3046875" style="1" customWidth="1"/>
-    <col min="8474" max="8704" width="9.23046875" style="1"/>
-    <col min="8705" max="8729" width="7.3046875" style="1" customWidth="1"/>
-    <col min="8730" max="8960" width="9.23046875" style="1"/>
-    <col min="8961" max="8985" width="7.3046875" style="1" customWidth="1"/>
-    <col min="8986" max="9216" width="9.23046875" style="1"/>
-    <col min="9217" max="9241" width="7.3046875" style="1" customWidth="1"/>
-    <col min="9242" max="9472" width="9.23046875" style="1"/>
-    <col min="9473" max="9497" width="7.3046875" style="1" customWidth="1"/>
-    <col min="9498" max="9728" width="9.23046875" style="1"/>
-    <col min="9729" max="9753" width="7.3046875" style="1" customWidth="1"/>
-    <col min="9754" max="9984" width="9.23046875" style="1"/>
-    <col min="9985" max="10009" width="7.3046875" style="1" customWidth="1"/>
-    <col min="10010" max="10240" width="9.23046875" style="1"/>
-    <col min="10241" max="10265" width="7.3046875" style="1" customWidth="1"/>
-    <col min="10266" max="10496" width="9.23046875" style="1"/>
-    <col min="10497" max="10521" width="7.3046875" style="1" customWidth="1"/>
-    <col min="10522" max="10752" width="9.23046875" style="1"/>
-    <col min="10753" max="10777" width="7.3046875" style="1" customWidth="1"/>
-    <col min="10778" max="11008" width="9.23046875" style="1"/>
-    <col min="11009" max="11033" width="7.3046875" style="1" customWidth="1"/>
-    <col min="11034" max="11264" width="9.23046875" style="1"/>
-    <col min="11265" max="11289" width="7.3046875" style="1" customWidth="1"/>
-    <col min="11290" max="11520" width="9.23046875" style="1"/>
-    <col min="11521" max="11545" width="7.3046875" style="1" customWidth="1"/>
-    <col min="11546" max="11776" width="9.23046875" style="1"/>
-    <col min="11777" max="11801" width="7.3046875" style="1" customWidth="1"/>
-    <col min="11802" max="12032" width="9.23046875" style="1"/>
-    <col min="12033" max="12057" width="7.3046875" style="1" customWidth="1"/>
-    <col min="12058" max="12288" width="9.23046875" style="1"/>
-    <col min="12289" max="12313" width="7.3046875" style="1" customWidth="1"/>
-    <col min="12314" max="12544" width="9.23046875" style="1"/>
-    <col min="12545" max="12569" width="7.3046875" style="1" customWidth="1"/>
-    <col min="12570" max="12800" width="9.23046875" style="1"/>
-    <col min="12801" max="12825" width="7.3046875" style="1" customWidth="1"/>
-    <col min="12826" max="13056" width="9.23046875" style="1"/>
-    <col min="13057" max="13081" width="7.3046875" style="1" customWidth="1"/>
-    <col min="13082" max="13312" width="9.23046875" style="1"/>
-    <col min="13313" max="13337" width="7.3046875" style="1" customWidth="1"/>
-    <col min="13338" max="13568" width="9.23046875" style="1"/>
-    <col min="13569" max="13593" width="7.3046875" style="1" customWidth="1"/>
-    <col min="13594" max="13824" width="9.23046875" style="1"/>
-    <col min="13825" max="13849" width="7.3046875" style="1" customWidth="1"/>
-    <col min="13850" max="14080" width="9.23046875" style="1"/>
-    <col min="14081" max="14105" width="7.3046875" style="1" customWidth="1"/>
-    <col min="14106" max="14336" width="9.23046875" style="1"/>
-    <col min="14337" max="14361" width="7.3046875" style="1" customWidth="1"/>
-    <col min="14362" max="14592" width="9.23046875" style="1"/>
-    <col min="14593" max="14617" width="7.3046875" style="1" customWidth="1"/>
-    <col min="14618" max="14848" width="9.23046875" style="1"/>
-    <col min="14849" max="14873" width="7.3046875" style="1" customWidth="1"/>
-    <col min="14874" max="15104" width="9.23046875" style="1"/>
-    <col min="15105" max="15129" width="7.3046875" style="1" customWidth="1"/>
-    <col min="15130" max="15360" width="9.23046875" style="1"/>
-    <col min="15361" max="15385" width="7.3046875" style="1" customWidth="1"/>
-    <col min="15386" max="15616" width="9.23046875" style="1"/>
-    <col min="15617" max="15641" width="7.3046875" style="1" customWidth="1"/>
-    <col min="15642" max="15872" width="9.23046875" style="1"/>
-    <col min="15873" max="15897" width="7.3046875" style="1" customWidth="1"/>
-    <col min="15898" max="16128" width="9.23046875" style="1"/>
-    <col min="16129" max="16153" width="7.3046875" style="1" customWidth="1"/>
-    <col min="16154" max="16384" width="9.23046875" style="1"/>
+    <col min="2" max="2" width="8.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="25" width="7.33203125" style="1" customWidth="1"/>
+    <col min="26" max="256" width="9.21875" style="1"/>
+    <col min="257" max="281" width="7.33203125" style="1" customWidth="1"/>
+    <col min="282" max="512" width="9.21875" style="1"/>
+    <col min="513" max="537" width="7.33203125" style="1" customWidth="1"/>
+    <col min="538" max="768" width="9.21875" style="1"/>
+    <col min="769" max="793" width="7.33203125" style="1" customWidth="1"/>
+    <col min="794" max="1024" width="9.21875" style="1"/>
+    <col min="1025" max="1049" width="7.33203125" style="1" customWidth="1"/>
+    <col min="1050" max="1280" width="9.21875" style="1"/>
+    <col min="1281" max="1305" width="7.33203125" style="1" customWidth="1"/>
+    <col min="1306" max="1536" width="9.21875" style="1"/>
+    <col min="1537" max="1561" width="7.33203125" style="1" customWidth="1"/>
+    <col min="1562" max="1792" width="9.21875" style="1"/>
+    <col min="1793" max="1817" width="7.33203125" style="1" customWidth="1"/>
+    <col min="1818" max="2048" width="9.21875" style="1"/>
+    <col min="2049" max="2073" width="7.33203125" style="1" customWidth="1"/>
+    <col min="2074" max="2304" width="9.21875" style="1"/>
+    <col min="2305" max="2329" width="7.33203125" style="1" customWidth="1"/>
+    <col min="2330" max="2560" width="9.21875" style="1"/>
+    <col min="2561" max="2585" width="7.33203125" style="1" customWidth="1"/>
+    <col min="2586" max="2816" width="9.21875" style="1"/>
+    <col min="2817" max="2841" width="7.33203125" style="1" customWidth="1"/>
+    <col min="2842" max="3072" width="9.21875" style="1"/>
+    <col min="3073" max="3097" width="7.33203125" style="1" customWidth="1"/>
+    <col min="3098" max="3328" width="9.21875" style="1"/>
+    <col min="3329" max="3353" width="7.33203125" style="1" customWidth="1"/>
+    <col min="3354" max="3584" width="9.21875" style="1"/>
+    <col min="3585" max="3609" width="7.33203125" style="1" customWidth="1"/>
+    <col min="3610" max="3840" width="9.21875" style="1"/>
+    <col min="3841" max="3865" width="7.33203125" style="1" customWidth="1"/>
+    <col min="3866" max="4096" width="9.21875" style="1"/>
+    <col min="4097" max="4121" width="7.33203125" style="1" customWidth="1"/>
+    <col min="4122" max="4352" width="9.21875" style="1"/>
+    <col min="4353" max="4377" width="7.33203125" style="1" customWidth="1"/>
+    <col min="4378" max="4608" width="9.21875" style="1"/>
+    <col min="4609" max="4633" width="7.33203125" style="1" customWidth="1"/>
+    <col min="4634" max="4864" width="9.21875" style="1"/>
+    <col min="4865" max="4889" width="7.33203125" style="1" customWidth="1"/>
+    <col min="4890" max="5120" width="9.21875" style="1"/>
+    <col min="5121" max="5145" width="7.33203125" style="1" customWidth="1"/>
+    <col min="5146" max="5376" width="9.21875" style="1"/>
+    <col min="5377" max="5401" width="7.33203125" style="1" customWidth="1"/>
+    <col min="5402" max="5632" width="9.21875" style="1"/>
+    <col min="5633" max="5657" width="7.33203125" style="1" customWidth="1"/>
+    <col min="5658" max="5888" width="9.21875" style="1"/>
+    <col min="5889" max="5913" width="7.33203125" style="1" customWidth="1"/>
+    <col min="5914" max="6144" width="9.21875" style="1"/>
+    <col min="6145" max="6169" width="7.33203125" style="1" customWidth="1"/>
+    <col min="6170" max="6400" width="9.21875" style="1"/>
+    <col min="6401" max="6425" width="7.33203125" style="1" customWidth="1"/>
+    <col min="6426" max="6656" width="9.21875" style="1"/>
+    <col min="6657" max="6681" width="7.33203125" style="1" customWidth="1"/>
+    <col min="6682" max="6912" width="9.21875" style="1"/>
+    <col min="6913" max="6937" width="7.33203125" style="1" customWidth="1"/>
+    <col min="6938" max="7168" width="9.21875" style="1"/>
+    <col min="7169" max="7193" width="7.33203125" style="1" customWidth="1"/>
+    <col min="7194" max="7424" width="9.21875" style="1"/>
+    <col min="7425" max="7449" width="7.33203125" style="1" customWidth="1"/>
+    <col min="7450" max="7680" width="9.21875" style="1"/>
+    <col min="7681" max="7705" width="7.33203125" style="1" customWidth="1"/>
+    <col min="7706" max="7936" width="9.21875" style="1"/>
+    <col min="7937" max="7961" width="7.33203125" style="1" customWidth="1"/>
+    <col min="7962" max="8192" width="9.21875" style="1"/>
+    <col min="8193" max="8217" width="7.33203125" style="1" customWidth="1"/>
+    <col min="8218" max="8448" width="9.21875" style="1"/>
+    <col min="8449" max="8473" width="7.33203125" style="1" customWidth="1"/>
+    <col min="8474" max="8704" width="9.21875" style="1"/>
+    <col min="8705" max="8729" width="7.33203125" style="1" customWidth="1"/>
+    <col min="8730" max="8960" width="9.21875" style="1"/>
+    <col min="8961" max="8985" width="7.33203125" style="1" customWidth="1"/>
+    <col min="8986" max="9216" width="9.21875" style="1"/>
+    <col min="9217" max="9241" width="7.33203125" style="1" customWidth="1"/>
+    <col min="9242" max="9472" width="9.21875" style="1"/>
+    <col min="9473" max="9497" width="7.33203125" style="1" customWidth="1"/>
+    <col min="9498" max="9728" width="9.21875" style="1"/>
+    <col min="9729" max="9753" width="7.33203125" style="1" customWidth="1"/>
+    <col min="9754" max="9984" width="9.21875" style="1"/>
+    <col min="9985" max="10009" width="7.33203125" style="1" customWidth="1"/>
+    <col min="10010" max="10240" width="9.21875" style="1"/>
+    <col min="10241" max="10265" width="7.33203125" style="1" customWidth="1"/>
+    <col min="10266" max="10496" width="9.21875" style="1"/>
+    <col min="10497" max="10521" width="7.33203125" style="1" customWidth="1"/>
+    <col min="10522" max="10752" width="9.21875" style="1"/>
+    <col min="10753" max="10777" width="7.33203125" style="1" customWidth="1"/>
+    <col min="10778" max="11008" width="9.21875" style="1"/>
+    <col min="11009" max="11033" width="7.33203125" style="1" customWidth="1"/>
+    <col min="11034" max="11264" width="9.21875" style="1"/>
+    <col min="11265" max="11289" width="7.33203125" style="1" customWidth="1"/>
+    <col min="11290" max="11520" width="9.21875" style="1"/>
+    <col min="11521" max="11545" width="7.33203125" style="1" customWidth="1"/>
+    <col min="11546" max="11776" width="9.21875" style="1"/>
+    <col min="11777" max="11801" width="7.33203125" style="1" customWidth="1"/>
+    <col min="11802" max="12032" width="9.21875" style="1"/>
+    <col min="12033" max="12057" width="7.33203125" style="1" customWidth="1"/>
+    <col min="12058" max="12288" width="9.21875" style="1"/>
+    <col min="12289" max="12313" width="7.33203125" style="1" customWidth="1"/>
+    <col min="12314" max="12544" width="9.21875" style="1"/>
+    <col min="12545" max="12569" width="7.33203125" style="1" customWidth="1"/>
+    <col min="12570" max="12800" width="9.21875" style="1"/>
+    <col min="12801" max="12825" width="7.33203125" style="1" customWidth="1"/>
+    <col min="12826" max="13056" width="9.21875" style="1"/>
+    <col min="13057" max="13081" width="7.33203125" style="1" customWidth="1"/>
+    <col min="13082" max="13312" width="9.21875" style="1"/>
+    <col min="13313" max="13337" width="7.33203125" style="1" customWidth="1"/>
+    <col min="13338" max="13568" width="9.21875" style="1"/>
+    <col min="13569" max="13593" width="7.33203125" style="1" customWidth="1"/>
+    <col min="13594" max="13824" width="9.21875" style="1"/>
+    <col min="13825" max="13849" width="7.33203125" style="1" customWidth="1"/>
+    <col min="13850" max="14080" width="9.21875" style="1"/>
+    <col min="14081" max="14105" width="7.33203125" style="1" customWidth="1"/>
+    <col min="14106" max="14336" width="9.21875" style="1"/>
+    <col min="14337" max="14361" width="7.33203125" style="1" customWidth="1"/>
+    <col min="14362" max="14592" width="9.21875" style="1"/>
+    <col min="14593" max="14617" width="7.33203125" style="1" customWidth="1"/>
+    <col min="14618" max="14848" width="9.21875" style="1"/>
+    <col min="14849" max="14873" width="7.33203125" style="1" customWidth="1"/>
+    <col min="14874" max="15104" width="9.21875" style="1"/>
+    <col min="15105" max="15129" width="7.33203125" style="1" customWidth="1"/>
+    <col min="15130" max="15360" width="9.21875" style="1"/>
+    <col min="15361" max="15385" width="7.33203125" style="1" customWidth="1"/>
+    <col min="15386" max="15616" width="9.21875" style="1"/>
+    <col min="15617" max="15641" width="7.33203125" style="1" customWidth="1"/>
+    <col min="15642" max="15872" width="9.21875" style="1"/>
+    <col min="15873" max="15897" width="7.33203125" style="1" customWidth="1"/>
+    <col min="15898" max="16128" width="9.21875" style="1"/>
+    <col min="16129" max="16153" width="7.33203125" style="1" customWidth="1"/>
+    <col min="16154" max="16384" width="9.21875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:24" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="36" t="s">
         <v>32</v>
       </c>
@@ -3834,7 +3827,7 @@
       <c r="W1" s="36"/>
       <c r="X1" s="37"/>
     </row>
-    <row r="2" spans="1:24" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:24" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="25" t="s">
         <v>33</v>
       </c>
@@ -3908,7 +3901,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>16</v>
       </c>
@@ -3982,7 +3975,7 @@
         <v>0.59</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>16</v>
       </c>
@@ -4053,7 +4046,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>16</v>
       </c>
@@ -4127,7 +4120,7 @@
         <v>0.61</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>16</v>
       </c>
@@ -4201,7 +4194,7 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
@@ -4275,7 +4268,7 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
@@ -4349,7 +4342,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
@@ -4423,7 +4416,7 @@
         <v>0.68</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -4497,7 +4490,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>16</v>
       </c>
@@ -4571,7 +4564,7 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>16</v>
       </c>
@@ -4645,7 +4638,7 @@
         <v>0.44</v>
       </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>16</v>
       </c>
@@ -4719,7 +4712,7 @@
         <v>0.66</v>
       </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>16</v>
       </c>
@@ -4793,7 +4786,7 @@
         <v>0.53</v>
       </c>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>16</v>
       </c>
@@ -4867,7 +4860,7 @@
         <v>0.62</v>
       </c>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>16</v>
       </c>
@@ -4941,7 +4934,7 @@
         <v>0.47</v>
       </c>
     </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>16</v>
       </c>
@@ -5015,7 +5008,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>20</v>
       </c>
@@ -5089,7 +5082,7 @@
         <v>0.59</v>
       </c>
     </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>20</v>
       </c>
@@ -5163,7 +5156,7 @@
         <v>0.64</v>
       </c>
     </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>20</v>
       </c>
@@ -5234,7 +5227,7 @@
         <v>0.44</v>
       </c>
     </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>20</v>
       </c>
@@ -5305,7 +5298,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
@@ -5373,7 +5366,7 @@
         <v>0.37</v>
       </c>
     </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>20</v>
       </c>
@@ -5447,7 +5440,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>20</v>
       </c>
@@ -5521,7 +5514,7 @@
         <v>0.39</v>
       </c>
     </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>20</v>
       </c>
@@ -5595,7 +5588,7 @@
         <v>0.48</v>
       </c>
     </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>20</v>
       </c>
@@ -5669,7 +5662,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>20</v>
       </c>
@@ -5743,7 +5736,7 @@
         <v>0.59</v>
       </c>
     </row>
-    <row r="28" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>20</v>
       </c>
@@ -5814,7 +5807,7 @@
         <v>0.51</v>
       </c>
     </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>20</v>
       </c>
@@ -5888,7 +5881,7 @@
         <v>0.49</v>
       </c>
     </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>20</v>
       </c>
@@ -5962,7 +5955,7 @@
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>20</v>
       </c>
@@ -6033,7 +6026,7 @@
         <v>0.54</v>
       </c>
     </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>20</v>
       </c>
@@ -6104,7 +6097,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="33" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>18</v>
       </c>
@@ -6178,7 +6171,7 @@
         <v>0.47</v>
       </c>
     </row>
-    <row r="34" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>18</v>
       </c>
@@ -6252,7 +6245,7 @@
         <v>0.47</v>
       </c>
     </row>
-    <row r="35" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>18</v>
       </c>
@@ -6323,7 +6316,7 @@
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="36" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>18</v>
       </c>
@@ -6394,7 +6387,7 @@
         <v>0.56000000000000005</v>
       </c>
     </row>
-    <row r="37" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>18</v>
       </c>
@@ -6468,7 +6461,7 @@
         <v>0.52</v>
       </c>
     </row>
-    <row r="38" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>18</v>
       </c>
@@ -6542,7 +6535,7 @@
         <v>0.38</v>
       </c>
     </row>
-    <row r="39" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>18</v>
       </c>
@@ -6616,7 +6609,7 @@
         <v>0.64</v>
       </c>
     </row>
-    <row r="40" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>18</v>
       </c>
@@ -6690,7 +6683,7 @@
         <v>0.53</v>
       </c>
     </row>
-    <row r="41" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>18</v>
       </c>
@@ -6764,7 +6757,7 @@
         <v>0.59</v>
       </c>
     </row>
-    <row r="42" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>18</v>
       </c>
@@ -6838,7 +6831,7 @@
         <v>0.47</v>
       </c>
     </row>
-    <row r="43" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>18</v>
       </c>
@@ -6912,7 +6905,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="44" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>18</v>
       </c>
@@ -6983,7 +6976,7 @@
         <v>0.64</v>
       </c>
     </row>
-    <row r="45" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>18</v>
       </c>
@@ -7054,7 +7047,7 @@
         <v>0.54</v>
       </c>
     </row>
-    <row r="46" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>18</v>
       </c>
@@ -7128,7 +7121,7 @@
         <v>0.44</v>
       </c>
     </row>
-    <row r="47" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>18</v>
       </c>
@@ -7202,7 +7195,7 @@
         <v>0.51</v>
       </c>
     </row>
-    <row r="48" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>35</v>
       </c>
@@ -7276,7 +7269,7 @@
         <v>0.46</v>
       </c>
     </row>
-    <row r="49" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>35</v>
       </c>
@@ -7347,7 +7340,7 @@
         <v>0.53</v>
       </c>
     </row>
-    <row r="50" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>35</v>
       </c>
@@ -7418,7 +7411,7 @@
         <v>0.42</v>
       </c>
     </row>
-    <row r="51" spans="1:24" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>35</v>
       </c>
@@ -7489,7 +7482,7 @@
         <v>0.46</v>
       </c>
     </row>
-    <row r="52" spans="1:24" ht="16.5" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:24" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>35</v>
       </c>
@@ -7572,14 +7565,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{536B55AF-236A-4ECC-9718-CC3AF22F8E66}">
   <dimension ref="B1:L8"/>
-  <sheetFormatPr defaultRowHeight="16" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="2:12" x14ac:dyDescent="0.4">
+    <row r="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B1" s="32" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="38" t="s">
         <v>37</v>
       </c>
@@ -7594,7 +7587,7 @@
       <c r="K3" s="38"/>
       <c r="L3" s="38"/>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="38"/>
       <c r="C4" s="38"/>
       <c r="D4" s="38"/>
@@ -7607,7 +7600,7 @@
       <c r="K4" s="38"/>
       <c r="L4" s="38"/>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="38"/>
       <c r="C5" s="38"/>
       <c r="D5" s="38"/>
@@ -7620,7 +7613,7 @@
       <c r="K5" s="38"/>
       <c r="L5" s="38"/>
     </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="39" t="s">
         <v>38</v>
       </c>
@@ -7635,7 +7628,7 @@
       <c r="K6" s="39"/>
       <c r="L6" s="39"/>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="39"/>
       <c r="C7" s="39"/>
       <c r="D7" s="39"/>
@@ -7648,7 +7641,7 @@
       <c r="K7" s="39"/>
       <c r="L7" s="39"/>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="39"/>
       <c r="C8" s="39"/>
       <c r="D8" s="39"/>

</xml_diff>